<commit_message>
Daily slate 2026-06-26 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-24.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-24.xlsx
@@ -503,13 +503,13 @@
         <v>13</v>
       </c>
       <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
         <v>8</v>
       </c>
-      <c r="F3" t="n">
-        <v>5</v>
-      </c>
       <c r="G3" t="n">
-        <v>61.5</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="E4" t="n">
+        <v>191</v>
+      </c>
+      <c r="F4" t="n">
         <v>185</v>
       </c>
-      <c r="F4" t="n">
-        <v>181</v>
-      </c>
       <c r="G4" t="n">
-        <v>50.5</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="5">
@@ -561,13 +561,13 @@
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="E7" t="n">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="F7" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="G7" t="n">
-        <v>48.8</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="8">
@@ -645,13 +645,13 @@
         <v>330</v>
       </c>
       <c r="E8" t="n">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="F8" t="n">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="G8" t="n">
-        <v>47.9</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="9">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E10" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F10" t="n">
         <v>67</v>
       </c>
       <c r="G10" t="n">
-        <v>73.59999999999999</v>
+        <v>73.8</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1391</v>
+        <v>1435</v>
       </c>
       <c r="E11" t="n">
-        <v>835</v>
+        <v>861</v>
       </c>
       <c r="F11" t="n">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="G11" t="n">
         <v>60</v>
@@ -758,13 +758,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E12" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F12" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G12" t="n">
         <v>69.8</v>
@@ -787,16 +787,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E13" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F13" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G13" t="n">
-        <v>47.6</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>433</v>
+        <v>447</v>
       </c>
       <c r="E14" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F14" t="n">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="G14" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="E15" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="F15" t="n">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="G15" t="n">
-        <v>21</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="16">
@@ -874,13 +874,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="E16" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F16" t="n">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="G16" t="n">
         <v>19.1</v>
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5178</v>
+        <v>5380</v>
       </c>
       <c r="E17" t="n">
-        <v>926</v>
+        <v>987</v>
       </c>
       <c r="F17" t="n">
-        <v>4252</v>
+        <v>4393</v>
       </c>
       <c r="G17" t="n">
-        <v>17.9</v>
+        <v>18.3</v>
       </c>
     </row>
   </sheetData>
@@ -1519,52 +1519,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>73.59999999999999</v>
+        <v>73.8</v>
       </c>
       <c r="C7" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D7" t="n">
         <v>60</v>
       </c>
       <c r="E7" t="n">
-        <v>1391</v>
+        <v>1435</v>
       </c>
       <c r="F7" t="n">
         <v>69.8</v>
       </c>
       <c r="G7" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H7" t="n">
-        <v>47.6</v>
+        <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="J7" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
       <c r="K7" t="n">
-        <v>433</v>
+        <v>447</v>
       </c>
       <c r="L7" t="n">
-        <v>21</v>
+        <v>21.4</v>
       </c>
       <c r="M7" t="n">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="N7" t="n">
         <v>19.1</v>
       </c>
       <c r="O7" t="n">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="P7" t="n">
-        <v>17.9</v>
+        <v>18.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>5178</v>
+        <v>5380</v>
       </c>
       <c r="R7" t="n">
         <v>55.9</v>
@@ -1573,37 +1573,37 @@
         <v>34</v>
       </c>
       <c r="T7" t="n">
-        <v>50.5</v>
+        <v>50.8</v>
       </c>
       <c r="U7" t="n">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>47.9</v>
+        <v>50.3</v>
       </c>
       <c r="Y7" t="n">
         <v>330</v>
       </c>
       <c r="Z7" t="n">
-        <v>61.5</v>
+        <v>38.5</v>
       </c>
       <c r="AA7" t="n">
         <v>13</v>
       </c>
       <c r="AB7" t="n">
-        <v>100</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AC7" t="n">
         <v>7</v>
       </c>
       <c r="AD7" t="n">
-        <v>48.8</v>
+        <v>49.8</v>
       </c>
       <c r="AE7" t="n">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="AF7" t="n">
         <v>55.4</v>

</xml_diff>